<commit_message>
added new hero counters
</commit_message>
<xml_diff>
--- a/archive/mobile_legends_heroes_updated_NEW.xlsx
+++ b/archive/mobile_legends_heroes_updated_NEW.xlsx
@@ -6,12 +6,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heroes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data-Input" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documentation - Computations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CounterCalculator" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LookupCalc" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ConditionValues" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heroes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data-Input" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documentation - Computations" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CounterCalculator" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LookupCalc" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -179,10 +180,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -468,6 +469,1238 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A174"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Aamon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Akai</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Aldous</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Alpha</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Alucard</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Angela</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Anti-Heal</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AoE CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AoE Damage</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Argus</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Arlott</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Atlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Aulus</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Aurora</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Badang</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Balmond</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Bane</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Barats</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Baxia</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Beatrix</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Belerick</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Benedetta</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Blood</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Brody</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bruno</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Burst</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Carmilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Cecilion</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Chang'e</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Chip</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Chou</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Cici</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Clint</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Cyclops</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Damage Reduction</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Dash/Blink</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Death Immunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Diggie</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>DPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Dyrroth</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Edith</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Esmeralda</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Estes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Execute</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Fanny</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Faramis</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Fighter</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Floryn</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Franco</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Fredrinn</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Freya</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Gatotkaca</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Global Dive</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Gloo</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Gord</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Granger</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Grock</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Guinevere</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Gusion</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Hanabi</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Hanzo</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Hard CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Harith</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Harley</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Hayabusa</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Healing</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Helcurt</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>High Mobility</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Hilda</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Hirara</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Hylos</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>I-Frame</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Irithel</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Ixia</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Jawhead</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Johnson</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Joy</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Julian</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Kadita</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Kagura</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Kaja</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Kalea</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Karina</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Karrie</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Khaleed</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Khufra</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Kimmy</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Lancelot</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Lapu-Lapu</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Layla</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Leomord</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Lesley</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Ling</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Lolita</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Lukas</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Lunox</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Luo Yi</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Lylia</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Mage</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Magic</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Mana</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Marcel</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Marksman</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Martis</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Masha</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Mathilda</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Melissa</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Minotaur</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Minsitthar</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Miya</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Mobility</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Morph</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Moskov</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Nana</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Natalia</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Natan</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Nolan</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Novaria</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Obsidia</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Odette</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Paquito</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Pharsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Phoveus</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Poke</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Popol and Kupa</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Rafaela</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Rage</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Remove CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Roger</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Ruby</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Saber</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Selena</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Shield</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Silvanna</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Soft CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Sora</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Stealth</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Summoner</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Sustain</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Suyou</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Tank</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Targeted CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Terizla</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Thamuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Tigreal</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>True Damage</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Uranus</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Vale</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Valentina</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Valir</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Vexana</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Vision</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Wanwan</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>X.Borg</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Xavier</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Yi Sun-shin</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Yin</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Yu Zhong</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Yve</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Zetian</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Zhask</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Zhuxin</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Zilong</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:R134"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
@@ -10478,7 +11711,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10939,14 +12172,14 @@
         </is>
       </c>
       <c r="D29" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>-25</v>
+        <v>-23</v>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Anti-mobility Fighter: Contempt/Soul Reaper marks and executes blink/dash divers who commit onto him.</t>
+          <t>Anti-mobility Fighter: Contempt/Soul Reaper marks and executes blink/dash divers who commit onto him. (Merged with overlapping Mobility/High Mobility rows below, averaged + tag-count adjustment to prevent triple-stacking)</t>
         </is>
       </c>
       <c r="I29" s="1" t="inlineStr">
@@ -10977,14 +12210,14 @@
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>-22</v>
+        <v>-23</v>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Punishes sustained-mobility assassins that must stay in his kit range to deal damage.</t>
+          <t>Punishes sustained-mobility assassins that must stay in his kit range to deal damage. (Same merged value as Dash/Blink row - only highest single match should apply per target)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -11010,14 +12243,14 @@
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>-14</v>
+        <v>-23</v>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>General mobility-tag matchup bonus for Phoveus.</t>
+          <t>General mobility-tag matchup bonus for Phoveus. (Merged value - use as fallback only if neither narrower tag applies)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -11109,14 +12342,14 @@
         </is>
       </c>
       <c r="D34" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>-18</v>
+        <v>-13</v>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Bouncing Ball cancels dashes/blinks mid-animation, hard-locking mobility divers.</t>
+          <t>Bouncing Ball and Skill 2 knock-up cancel dashes/blinks mid-animation, hard-locking mobility divers. (Duplicate rows merged and averaged with tag-count adjustment)</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -11142,14 +12375,14 @@
         </is>
       </c>
       <c r="D35" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>-15</v>
+        <v>-13</v>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Sturdiness plus Charging Roar punish sustained-mobility assassins.</t>
+          <t>Sturdiness plus Charging Roar punish sustained-mobility assassins. (Duplicate rows merged and averaged with tag-count adjustment)</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -11406,7 +12639,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Slow/root from Camellia Sword denies Fanny's cable-swing kiting window.</t>
+          <t>Camellia's Ring root denies Fanny's cable-swing kiting window. (Corrected: kit is Smart Heal / Camellia's Ring / Punishment of Nature, not 'Camellia Sword')</t>
         </is>
       </c>
     </row>
@@ -11518,7 +12751,7 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Shield-and-reflect kit is disproportionately strong vs magic burst (new DamageType rule type).</t>
+          <t>Shield-and-reflect kit is disproportionately strong vs magic burst.</t>
         </is>
       </c>
     </row>
@@ -11546,7 +12779,7 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Peel/shield kit is disproportionately strong protecting/denying squishy marksman targets (new Role rule type).</t>
+          <t>Peel/shield kit is disproportionately strong protecting/denying squishy marksman targets.</t>
         </is>
       </c>
     </row>
@@ -11595,14 +12828,14 @@
         </is>
       </c>
       <c r="D51" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>-12</v>
+        <v>-13</v>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>High-damage charge combos punish sustained-mobility heroes.</t>
+          <t>High-damage charge combos punish sustained-mobility heroes. (Merged with overlapping Dash/Blink row, averaged with tag-count adjustment)</t>
         </is>
       </c>
     </row>
@@ -11623,14 +12856,14 @@
         </is>
       </c>
       <c r="D52" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>-10</v>
+        <v>-13</v>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Mobility skill and CC chain disrupt dash-reliant divers.</t>
+          <t>Mobility skill and CC chain disrupt dash-reliant divers. (Merged value - only highest single match should apply per target)</t>
         </is>
       </c>
     </row>
@@ -11714,7 +12947,7 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Passive deals percent Max HP True Damage shredding tank HP pools.</t>
+          <t>Passive converts physical attack into true damage on-hit, letting her out-scale defense-stacking tanks. (Corrected: not a flat percent-Max-HP effect)</t>
         </is>
       </c>
     </row>
@@ -11749,7 +12982,7 @@
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Khufra</t>
+          <t>Hilda</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -11759,175 +12992,175 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>High Mobility</t>
+          <t>Burst</t>
         </is>
       </c>
       <c r="D57" s="4" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>-4</v>
+        <v>-14</v>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Bouncing Ball and Charging Roar interrupt high-mobility assassins.</t>
+          <t>Bush-regen burst punishes burst heroes who overextend.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Khufra</t>
+          <t>Saber</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Dash/Blink</t>
+          <t>Assassin</t>
         </is>
       </c>
       <c r="D58" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>-5</v>
+        <v>-10</v>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Skill 2 knocks up enemies dashing through Khufra.</t>
+          <t>Point-and-click airborne kills squishy assassin divers.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Hilda</t>
+          <t>Harley</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Burst</t>
+          <t>Hanzo</t>
         </is>
       </c>
       <c r="D59" s="4" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E59" s="4" t="n">
-        <v>-14</v>
+        <v>-20</v>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Bush-regen burst punishes burst heroes who overextend.</t>
+          <t>Lock-on ring ultimate deletes Hanzo before he can escape.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>Saber</t>
+          <t>Angela</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Assassin</t>
+          <t>Harley</t>
         </is>
       </c>
       <c r="D60" s="4" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>-10</v>
+        <v>-18</v>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Point-and-click airborne kills squishy assassin divers.</t>
+          <t>Slow and root deny Harley teleport-in burst window, preventing burst kill setup on Harley.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>Harley</t>
+          <t>Baxia</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Hanzo</t>
+          <t>Healing</t>
         </is>
       </c>
       <c r="D61" s="4" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>-20</v>
+        <v>-12</v>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Lock-on ring ultimate deletes Hanzo before he can escape.</t>
+          <t>Passive reduces enemy healing and shield output, wearing down sustain/heal comps.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Angela</t>
+          <t>Lunox</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Harley</t>
+          <t>Tank</t>
         </is>
       </c>
       <c r="D62" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E62" s="4" t="n">
-        <v>-18</v>
+        <v>-12</v>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Slow and root deny Harley teleport-in burst window.</t>
+          <t>Dark Form converts Magic Pen into percent HP magic damage.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Esmeralda</t>
+          <t>Dyrroth</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Tank</t>
         </is>
       </c>
       <c r="D63" s="4" t="n">
@@ -11938,14 +13171,14 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Passive converts enemy shields into her own health.</t>
+          <t>Skill 2 shreds Physical Defense for early trade wins.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Baxia</t>
+          <t>Dyrroth</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -11955,81 +13188,81 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Healing</t>
+          <t>Sustain</t>
         </is>
       </c>
       <c r="D64" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>-12</v>
+        <v>-8</v>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Passive reduces enemy healing and shield output by 50%.</t>
+          <t>Defense shred negates sustain-tank regen.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Lunox</t>
+          <t>Minsitthar</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Tank</t>
+          <t>Dash/Blink</t>
         </is>
       </c>
       <c r="D65" s="4" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>-12</v>
+        <v>-21</v>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Dark Form converts Magic Pen into percent HP magic damage.</t>
+          <t>Ultimate disables dash, blink, and mobility skills. (Merged with overlapping High Mobility row, averaged with tag-count adjustment)</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>Dyrroth</t>
+          <t>Minsitthar</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Tank</t>
+          <t>High Mobility</t>
         </is>
       </c>
       <c r="D66" s="4" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E66" s="4" t="n">
-        <v>-10</v>
+        <v>-21</v>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Skill 2 shreds up to 75% Physical Defense for early trade wins.</t>
+          <t>King Calling denies wall-climbing and continuous mobility. (Merged value - only highest single match should apply per target)</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Dyrroth</t>
+          <t>Kaja</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -12039,25 +13272,25 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Sustain</t>
+          <t>Dash/Blink</t>
         </is>
       </c>
       <c r="D67" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E67" s="4" t="n">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Defense shred negates sustain-tank regen.</t>
+          <t>Suppression drags blink divers into the team.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Minsitthar</t>
+          <t>Belerick</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -12067,53 +13300,53 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Dash/Blink</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="D68" s="4" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E68" s="4" t="n">
-        <v>-20</v>
+        <v>-12</v>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Ultimate disables dash, blink, and mobility skills.</t>
+          <t>Passive thorns reflect Max HP damage at attack-speed heroes.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Minsitthar</t>
+          <t>Belerick</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>High Mobility</t>
+          <t>Marksman</t>
         </is>
       </c>
       <c r="D69" s="4" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E69" s="4" t="n">
-        <v>-18</v>
+        <v>-8</v>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>King Calling denies wall-climbing and continuous mobility.</t>
+          <t>Thorned retaliation punishes sustained marksman output.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>Kaja</t>
+          <t>Wanwan</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -12123,25 +13356,25 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Dash/Blink</t>
+          <t>Targeted CC</t>
         </is>
       </c>
       <c r="D70" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E70" s="4" t="n">
         <v>-10</v>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Suppression drags blink divers into the team.</t>
+          <t>Skill 2 Purify removes point-and-click stuns.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>Belerick</t>
+          <t>Wanwan</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -12151,53 +13384,53 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>DPS</t>
+          <t>Hard CC</t>
         </is>
       </c>
       <c r="D71" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E71" s="4" t="n">
-        <v>-12</v>
+        <v>-8</v>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Passive thorns reflect Max HP damage at attack-speed heroes.</t>
+          <t>Built-in CC cleanse denies hard-engage ults.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>Belerick</t>
+          <t>Valir</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Marksman</t>
+          <t>Dash/Blink</t>
         </is>
       </c>
       <c r="D72" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E72" s="4" t="n">
-        <v>-8</v>
+        <v>-12</v>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>Thorned retaliation punishes sustained marksman output.</t>
+          <t>Continuous knockbacks keep melee divers at distance.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>Wanwan</t>
+          <t>Valir</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -12207,25 +13440,25 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Targeted CC</t>
+          <t>Sustain</t>
         </is>
       </c>
       <c r="D73" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E73" s="4" t="n">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>Skill 2 Purify removes point-and-click stuns.</t>
+          <t>Burning damage kites sustain brawlers before they close.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>Wanwan</t>
+          <t>Martis</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -12246,14 +13479,14 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Built-in CC cleanse denies hard-engage ults.</t>
+          <t>Skill 2 grants full CC immunity during execution.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>Valir</t>
+          <t>Martis</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -12263,25 +13496,25 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Dash/Blink</t>
+          <t>AoE CC</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E75" t="n">
-        <v>-12</v>
+        <v>-6</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Continuous knockbacks keep melee divers at distance.</t>
+          <t>CC immunity ignores multi-target crowd control.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>Valir</t>
+          <t>Akai</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -12291,7 +13524,7 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Sustain</t>
+          <t>AoE Damage</t>
         </is>
       </c>
       <c r="D76" s="4" t="n">
@@ -12302,14 +13535,14 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Burning damage kites sustain brawlers before they close.</t>
+          <t>Ultimate knockback interrupts channeled area ults.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>Martis</t>
+          <t>Irithel</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -12319,7 +13552,7 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Hard CC</t>
+          <t>Poke</t>
         </is>
       </c>
       <c r="D77" s="4" t="n">
@@ -12330,14 +13563,14 @@
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Skill 2 grants full CC immunity during execution.</t>
+          <t>Move-while-attacking circles directional skillshots.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>Martis</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
@@ -12347,35 +13580,35 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>AoE CC</t>
+          <t>Summoner</t>
         </is>
       </c>
       <c r="D78" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E78" s="4" t="n">
-        <v>-6</v>
+        <v>-10</v>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>CC immunity ignores multi-target crowd control.</t>
+          <t>Passive clone gains extra proc targets against summoner comps. (Corrected: ultimate mirrors enemy hero attacks, not summon-triggered stacking; value reduced to reflect thinner justification)</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Akai</t>
+          <t>Lesley</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>AoE Damage</t>
+          <t>Marksman</t>
         </is>
       </c>
       <c r="D79" s="4" t="n">
@@ -12386,14 +13619,14 @@
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Ultimate knockback interrupts channeled area ults.</t>
+          <t>Stealth range and True Damage poke down short-range MMs.</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>Irithel</t>
+          <t>Lesley</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -12403,53 +13636,53 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Poke</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="D80" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E80" s="4" t="n">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Move-while-attacking circles directional skillshots.</t>
+          <t>Invisible repositioning punishes sustained DPS heroes.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Natan</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Summoner</t>
+          <t>Tank</t>
         </is>
       </c>
       <c r="D81" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E81" s="4" t="n">
-        <v>-14</v>
+        <v>-10</v>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Ultimate hits clones triggering Demon Hunter Sword stacks.</t>
+          <t>Bonus magic power scaling from physical attack lets him bypass armor-stacking tanks. (Corrected: hybrid on-hit scaling, not a Pen-conversion mechanic)</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>Lesley</t>
+          <t>Brody</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
@@ -12470,52 +13703,52 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>Stealth range and True Damage poke down short-range MMs.</t>
+          <t>Passive mark locking executes squishy backliners.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>Lesley</t>
+          <t>Brody</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>DPS</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="D83" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E83" s="4" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>Invisible repositioning punishes sustained DPS heroes.</t>
+          <t>Physical burst deletes immobile mages.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>Natan</t>
+          <t>Eudora</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Tank</t>
+          <t>High Mobility</t>
         </is>
       </c>
       <c r="D84" s="4" t="n">
@@ -12526,52 +13759,52 @@
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>Converts Physical Pen into Magic Pen bypassing armor.</t>
+          <t>Point-and-click stun chain freezes fast assassins.</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Brody</t>
+          <t>Aurora</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Marksman</t>
+          <t>High Mobility</t>
         </is>
       </c>
       <c r="D85" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E85" s="4" t="n">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>Passive mark locking executes squishy backliners.</t>
+          <t>AoE freeze punishes high-mobility divers.</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>Brody</t>
+          <t>Kagura</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Mage</t>
+          <t>Targeted CC</t>
         </is>
       </c>
       <c r="D86" s="4" t="n">
@@ -12582,14 +13815,14 @@
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>Physical burst deletes immobile mages.</t>
+          <t>Umbrella purge removes debuffs and grants dash.</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>Eudora</t>
+          <t>Zhask</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
@@ -12599,25 +13832,25 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>High Mobility</t>
+          <t>Burst</t>
         </is>
       </c>
       <c r="D87" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E87" s="4" t="n">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Point-and-click stun chain freezes fast assassins.</t>
+          <t>Nightmarish Spawn disjoints targeted burst spells.</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>Aurora</t>
+          <t>Zhask</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
@@ -12627,25 +13860,25 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>High Mobility</t>
+          <t>Targeted CC</t>
         </is>
       </c>
       <c r="D88" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E88" s="4" t="n">
-        <v>-10</v>
+        <v>-6</v>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>AoE freeze punishes high-mobility divers.</t>
+          <t>Spawn body-blocks point-and-click control.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>Kagura</t>
+          <t>Kadita</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
@@ -12655,7 +13888,7 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Targeted CC</t>
+          <t>Hard CC</t>
         </is>
       </c>
       <c r="D89" s="4" t="n">
@@ -12666,14 +13899,14 @@
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>Umbrella purge removes debuffs and grants dash.</t>
+          <t>Skill 1 grants CC immunity on initiation.</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>Zhask</t>
+          <t>Kadita</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
@@ -12683,25 +13916,25 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Burst</t>
+          <t>Dash/Blink</t>
         </is>
       </c>
       <c r="D90" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E90" s="4" t="n">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>Nightmarish Spawn disjoints targeted burst spells.</t>
+          <t>CC immunity lets her dive through disengage blinks.</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>Zhask</t>
+          <t>Gord</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
@@ -12711,25 +13944,25 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Targeted CC</t>
+          <t>Sustain</t>
         </is>
       </c>
       <c r="D91" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E91" s="4" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>Spawn body-blocks point-and-click control.</t>
+          <t>True Damage melts sustain tanks before they reach backline.</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>Kadita</t>
+          <t>Gord</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
@@ -12739,53 +13972,53 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Hard CC</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="D92" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E92" s="4" t="n">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>Skill 1 grants CC immunity on initiation.</t>
+          <t>Skill 1 poke burns through shields from safe distance.</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>Kadita</t>
+          <t>Harley</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Dash/Blink</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="D93" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E93" s="4" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>CC immunity lets her dive through disengage blinks.</t>
+          <t>Teleport and lock-on ultimate dive static mages.</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>Gord</t>
+          <t>Terizla</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
@@ -12795,7 +14028,7 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Sustain</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="D94" s="4" t="n">
@@ -12806,14 +14039,14 @@
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>True Damage melts sustain tanks before they reach backline.</t>
+          <t>Passive damage reduction wins long trades vs sustained DPS.</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>Gord</t>
+          <t>X.Borg</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
@@ -12823,53 +14056,53 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Sustain</t>
         </is>
       </c>
       <c r="D95" s="4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E95" s="4" t="n">
-        <v>-6</v>
+        <v>-12</v>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>Skill 1 poke burns through shields from safe distance.</t>
+          <t>Skill 1 True Damage ignores armor and lifesteal.</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>Harley</t>
+          <t>X.Borg</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>Mage</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="D96" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E96" s="4" t="n">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>Teleport and lock-on ultimate dive static mages.</t>
+          <t>True Damage bypasses shield mechanics.</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>Terizla</t>
+          <t>Thamuz</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
@@ -12890,52 +14123,52 @@
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Passive damage reduction wins long trades vs sustained DPS.</t>
+          <t>Lava True Damage and regen out-sustain basic-attack brawlers.</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>X.Borg</t>
+          <t>Carmilla</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Hero</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Sustain</t>
+          <t>Gloo</t>
         </is>
       </c>
       <c r="D98" s="4" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E98" s="4" t="n">
-        <v>-12</v>
+        <v>-16</v>
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>Skill 1 True Damage ignores armor and lifesteal.</t>
+          <t>Ultimate links Gloo clones to chain entire team.</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>X.Borg</t>
+          <t>Yu Zhong</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Marksman</t>
         </is>
       </c>
       <c r="D99" s="4" t="n">
@@ -12946,80 +14179,80 @@
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>True Damage bypasses shield mechanics.</t>
+          <t>Black Dragon bypasses frontliners to hit backline.</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>Thamuz</t>
+          <t>Yu Zhong</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Tag</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>DPS</t>
+          <t>Mage</t>
         </is>
       </c>
       <c r="D100" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E100" s="4" t="n">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>Lava True Damage and regen out-sustain basic-attack brawlers.</t>
+          <t>Flight and CC immunity dive immobile mages.</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>Carmilla</t>
+          <t>Arlott</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Gloo</t>
+          <t>Dash/Blink</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E101" t="n">
-        <v>-16</v>
+        <v>-10</v>
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>Ultimate links Gloo clones to chain entire team.</t>
+          <t>Passive grants Skill 2 dash resets vs mobile heroes.</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>Yu Zhong</t>
+          <t>Benedetta</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>Marksman</t>
+          <t>Hard CC</t>
         </is>
       </c>
       <c r="D102" s="4" t="n">
@@ -13030,42 +14263,42 @@
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Black Dragon bypasses frontliners to hit backline.</t>
+          <t>Skill 2 grants CC immunity and reflects stuns.</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>Yu Zhong</t>
+          <t>Vexana</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Tag</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Mage</t>
+          <t>Summoner</t>
         </is>
       </c>
       <c r="D103" s="4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E103" s="4" t="n">
-        <v>-10</v>
+        <v>-14</v>
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>Flight and CC immunity dive immobile mages.</t>
+          <t>Passive causes summons to explode for chain AoE.</t>
         </is>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>Arlott</t>
+          <t>Lancelot</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
@@ -13075,7 +14308,7 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Dash/Blink</t>
+          <t>Summoner</t>
         </is>
       </c>
       <c r="D104" s="4" t="n">
@@ -13086,14 +14319,14 @@
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>Passive grants Skill 2 dash resets vs mobile heroes.</t>
+          <t>Summons create extra hitboxes for Skill 1 resets.</t>
         </is>
       </c>
     </row>
     <row r="105" ht="15" customHeight="1">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>Benedetta</t>
+          <t>Fanny</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
@@ -13103,7 +14336,7 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Hard CC</t>
+          <t>Summoner</t>
         </is>
       </c>
       <c r="D105" s="4" t="n">
@@ -13114,14 +14347,14 @@
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>Skill 2 grants CC immunity and reflects stuns.</t>
+          <t>Extra targets grant cable energy and stacks.</t>
         </is>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>Vexana</t>
+          <t>Masha</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
@@ -13131,25 +14364,25 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Summoner</t>
+          <t>Burst</t>
         </is>
       </c>
       <c r="D106" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E106" s="4" t="n">
-        <v>-14</v>
+        <v>-11</v>
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>Passive causes summons to explode for chain AoE.</t>
+          <t>Three HP bars absorb burst combos, leaving Masha alive. (Bumped slightly to match comparable burst-absorption value on Hylos)</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>Lancelot</t>
+          <t>Masha</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
@@ -13159,25 +14392,25 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Summoner</t>
+          <t>Targeted CC</t>
         </is>
       </c>
       <c r="D107" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E107" s="4" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>Summons create extra hitboxes for Skill 1 resets.</t>
+          <t>HP bars absorb point-and-click burst rotations. (Bumped slightly for consistency with Burst row)</t>
         </is>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>Fanny</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
@@ -13187,25 +14420,25 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Summoner</t>
+          <t>Global Dive</t>
         </is>
       </c>
       <c r="D108" s="4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E108" s="4" t="n">
-        <v>-10</v>
+        <v>-18</v>
       </c>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>Extra targets grant cable energy and stacks.</t>
+          <t>Abyssal Pull ultimate drags and binds the entire enemy team, hard-countering global-dive engage comps before they can scatter.</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15" customHeight="1">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>Masha</t>
+          <t>Grock</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
@@ -13215,25 +14448,25 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Burst</t>
+          <t>Dash/Blink</t>
         </is>
       </c>
       <c r="D109" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E109" s="4" t="n">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>Three HP bars absorb burst combos, leaving Masha alive.</t>
+          <t>Boulder Toss wall physically blocks dash/blink paths, denying clean engage routes for divers.</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15" customHeight="1">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>Masha</t>
+          <t>Estes</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
@@ -13243,156 +14476,496 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Targeted CC</t>
+          <t>Burst</t>
         </is>
       </c>
       <c r="D110" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E110" s="4" t="n">
-        <v>-6</v>
+        <v>-8</v>
       </c>
       <c r="F110" s="3" t="inlineStr">
         <is>
-          <t>HP bars absorb point-and-click burst rotations.</t>
+          <t>Passive AoE regeneration to the whole team blunts coordinated burst-kill attempts.</t>
         </is>
       </c>
     </row>
     <row r="111" ht="15" customHeight="1">
-      <c r="A111" s="4" t="n"/>
-      <c r="B111" s="4" t="n"/>
-      <c r="C111" s="4" t="n"/>
-      <c r="D111" s="4" t="n"/>
-      <c r="E111" s="4" t="n"/>
-      <c r="F111" s="3" t="n"/>
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>Floryn</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>Burst</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E111" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>Ultimate bonds to an ally with heal-over-time and mitigation, denying burst execution windows on the carry.</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="15" customHeight="1">
-      <c r="A112" s="4" t="n"/>
-      <c r="B112" s="4" t="n"/>
-      <c r="C112" s="4" t="n"/>
-      <c r="D112" s="4" t="n"/>
-      <c r="E112" s="4" t="n"/>
-      <c r="F112" s="3" t="n"/>
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t>Nolan</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>Sustain</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E112" s="4" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>Void Strike's true-damage proc ignores defense and lifesteal, wearing down sustain-heavy opponents over extended trades.</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="15" customHeight="1">
-      <c r="A113" s="4" t="n"/>
-      <c r="B113" s="4" t="n"/>
-      <c r="C113" s="4" t="n"/>
-      <c r="D113" s="4" t="n"/>
-      <c r="E113" s="4" t="n"/>
-      <c r="F113" s="3" t="n"/>
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>Yin</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>Tank</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E113" s="4" t="n">
+        <v>-12</v>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>Passive true-damage marks stack up over a fight, shredding tank HP pools that scale purely on defense.</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="15" customHeight="1">
-      <c r="A114" s="4" t="n"/>
-      <c r="B114" s="4" t="n"/>
-      <c r="C114" s="4" t="n"/>
-      <c r="D114" s="4" t="n"/>
-      <c r="E114" s="4" t="n"/>
-      <c r="F114" s="3" t="n"/>
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>Valentina</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C114" s="4" t="inlineStr">
+        <is>
+          <t>Mage</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E114" s="4" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>Ultimate copies an enemy mage's own ultimate, turning their signature burst tool directly against them.</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="15" customHeight="1">
-      <c r="A115" s="4" t="n"/>
-      <c r="B115" s="4" t="n"/>
-      <c r="C115" s="4" t="n"/>
-      <c r="D115" s="4" t="n"/>
-      <c r="E115" s="4" t="n"/>
-      <c r="F115" s="3" t="n"/>
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>Joy</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>Dash/Blink</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E115" s="4" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>Resonating Point's mark-and-dash chain lets her reposition through and punish melee divers who commit onto her.</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="15" customHeight="1">
-      <c r="A116" s="4" t="n"/>
-      <c r="B116" s="4" t="n"/>
-      <c r="C116" s="4" t="n"/>
-      <c r="D116" s="4" t="n"/>
-      <c r="E116" s="4" t="n"/>
-      <c r="F116" s="3" t="n"/>
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>Barats</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>Dash/Blink</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E116" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>Charge and grapple mechanics yank dash-committed divers off their intended path.</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="15" customHeight="1">
-      <c r="A117" s="4" t="n"/>
-      <c r="B117" s="4" t="n"/>
-      <c r="C117" s="4" t="n"/>
-      <c r="D117" s="4" t="n"/>
-      <c r="E117" s="4" t="n"/>
-      <c r="F117" s="3" t="n"/>
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>Novaria</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>Marksman</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E117" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>Illusion clone poke and true-damage marks whittle down squishy marksmen from range before they can retaliate.</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="15" customHeight="1">
-      <c r="A118" s="4" t="n"/>
-      <c r="B118" s="4" t="n"/>
-      <c r="C118" s="4" t="n"/>
-      <c r="D118" s="4" t="n"/>
-      <c r="E118" s="4" t="n"/>
-      <c r="F118" s="3" t="n"/>
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t>Tigreal</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>Mage</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E118" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>Implosion's knock-up and displacement punish immobile backline mages who get caught out of position.</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="15" customHeight="1">
-      <c r="A119" s="4" t="n"/>
-      <c r="B119" s="4" t="n"/>
-      <c r="C119" s="4" t="n"/>
-      <c r="D119" s="4" t="n"/>
-      <c r="E119" s="4" t="n"/>
-      <c r="F119" s="3" t="n"/>
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>Julian</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>High Mobility</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E119" s="4" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>Mark-fueled movement speed and dash let him stick to and run down sustained-mobility divers.</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="15" customHeight="1">
-      <c r="A120" s="4" t="n"/>
-      <c r="B120" s="4" t="n"/>
-      <c r="C120" s="4" t="n"/>
-      <c r="D120" s="4" t="n"/>
-      <c r="E120" s="4" t="n"/>
-      <c r="F120" s="3" t="n"/>
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>Lukas</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>Marksman</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E120" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>Burst combo plus innate mobility deletes squishy marksmen before they can kite to safety.</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="15" customHeight="1">
-      <c r="A121" s="4" t="n"/>
-      <c r="B121" s="4" t="n"/>
-      <c r="C121" s="4" t="n"/>
-      <c r="D121" s="4" t="n"/>
-      <c r="E121" s="4" t="n"/>
-      <c r="F121" s="3" t="n"/>
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>Silvanna</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>Sustain</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E121" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>Judgment of Talas execute damage scales off missing HP, punishing sustain heroes who try to outlast her in prolonged trades.</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="15" customHeight="1">
-      <c r="A122" s="4" t="n"/>
-      <c r="B122" s="4" t="n"/>
-      <c r="C122" s="4" t="n"/>
-      <c r="D122" s="4" t="n"/>
-      <c r="E122" s="4" t="n"/>
-      <c r="F122" s="3" t="n"/>
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>Aulus</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>Sustain</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E122" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F122" s="3" t="inlineStr">
+        <is>
+          <t>Passive stacking rewards prolonged engagements, letting him out-trade sustain-heavy opponents the longer a fight runs.</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="15" customHeight="1">
-      <c r="A123" s="4" t="n"/>
-      <c r="B123" s="4" t="n"/>
-      <c r="C123" s="4" t="n"/>
-      <c r="D123" s="4" t="n"/>
-      <c r="E123" s="4" t="n"/>
-      <c r="F123" s="3" t="n"/>
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>Kimmy</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>Poke</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E123" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>Passive slow-immunity and hybrid damage switching let her out-range and out-poke rival poke mages.</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="15" customHeight="1">
-      <c r="A124" s="4" t="n"/>
-      <c r="B124" s="4" t="n"/>
-      <c r="C124" s="4" t="n"/>
-      <c r="D124" s="4" t="n"/>
-      <c r="E124" s="4" t="n"/>
-      <c r="F124" s="3" t="n"/>
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>Popol and Kupa</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>Poke</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E124" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>Totem zone denial and long-range traps contest space and out-position poke compositions.</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="15" customHeight="1">
-      <c r="A125" s="4" t="n"/>
-      <c r="B125" s="4" t="n"/>
-      <c r="C125" s="4" t="n"/>
-      <c r="D125" s="4" t="n"/>
-      <c r="E125" s="4" t="n"/>
-      <c r="F125" s="3" t="n"/>
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>Beatrix</t>
+        </is>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>Mage</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E125" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>Weapon-swap burst combo (Renner into Wesker) deletes low-HP mages before they can retaliate.</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="15" customHeight="1">
-      <c r="A126" s="4" t="n"/>
-      <c r="B126" s="4" t="n"/>
-      <c r="C126" s="4" t="n"/>
-      <c r="D126" s="4" t="n"/>
-      <c r="E126" s="4" t="n"/>
-      <c r="F126" s="3" t="n"/>
+      <c r="A126" s="4" t="inlineStr">
+        <is>
+          <t>Yve</t>
+        </is>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t>Poke</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E126" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>Zone-control burst outranges and out-damages rival poke mages contesting the same lane space.</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="15" customHeight="1">
-      <c r="A127" s="4" t="n"/>
-      <c r="B127" s="4" t="n"/>
-      <c r="C127" s="4" t="n"/>
-      <c r="D127" s="4" t="n"/>
-      <c r="E127" s="4" t="n"/>
-      <c r="F127" s="3" t="n"/>
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>Ixia</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>Mage</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E127" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>Rapid-fire piercing shots delete squishy, immobile mages before they can complete their cast animation.</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="15" customHeight="1">
       <c r="A128" s="4" t="n"/>
@@ -25946,10 +27519,15 @@
     <mergeCell ref="A188:E188"/>
     <mergeCell ref="A17:H17"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="B29:B128" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid type" error="Must be &quot;Tag&quot; or &quot;Hero&quot;." type="list">
-      <formula1>"Tag,Hero,Role,DamageType,Resource"</formula1>
-      <formula2>0</formula2>
+  <dataValidations count="3">
+    <dataValidation sqref="A29:A128" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid hero" error="Pick a hero name from the list." type="list">
+      <formula1>=Heroes!$B$2:$B$134</formula1>
+    </dataValidation>
+    <dataValidation sqref="B29:B128" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid type" error="Pick Tag, Hero, Role, DamageType, or Resource." type="list">
+      <formula1>Tag,Hero,Role,DamageType,Resource</formula1>
+    </dataValidation>
+    <dataValidation sqref="C29:C128" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick a valid condition value from the list." type="list">
+      <formula1>=_ConditionValues!$A$1:$A$174</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -25957,7 +27535,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25984,7 +27562,7 @@
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>1. WORKBOOK MAP</t>
         </is>
@@ -26026,7 +27604,7 @@
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>2. WHAT "TAGS" MEANS IN THIS MODEL</t>
         </is>
@@ -26040,7 +27618,7 @@
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>3. THE COUNTER SCORE FORMULA</t>
         </is>
@@ -26068,7 +27646,7 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>Formula: MAX( RoleMatrix[Attacker.role -&gt; Defender.role] , RoleMatrix[Attacker.role2 -&gt; Defender.role] ) x role_mult</t>
         </is>
@@ -26089,7 +27667,7 @@
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>Formula: ((Attacker.offense + Attacker.ability_effects) / 2 − Defender.durability) x burst_mult</t>
         </is>
@@ -26110,7 +27688,7 @@
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="20" t="inlineStr">
         <is>
           <t>Formula: IF( (Attacker.difficulty − Defender.difficulty) &gt; 20 , (Attacker.difficulty − Defender.difficulty) x diff_mult , 0 )</t>
         </is>
@@ -26131,7 +27709,7 @@
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="21" t="inlineStr">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>Formula: IF(Attacker.damage_type = "Mixed", dmgtype_mixed, IF(Attacker.damage_type = Defender.damage_type, dmgtype_same, dmgtype_diff))</t>
         </is>
@@ -26152,7 +27730,7 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="21" t="inlineStr">
+      <c r="A35" s="20" t="inlineStr">
         <is>
           <t>Formula: (Attacker.spike_order − Defender.spike_order) x spike_mult</t>
         </is>
@@ -26173,7 +27751,7 @@
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="21" t="inlineStr">
+      <c r="A38" s="20" t="inlineStr">
         <is>
           <t>Formula: MAX of up to 4 lookups — (Attacker.style1 or style2) vs (Defender.style1 or style2) — read from the Style/Tag Interaction Matrix (Data-Input Block 5), x style_mult (default 5).</t>
         </is>
@@ -26243,7 +27821,7 @@
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="20" t="inlineStr">
+      <c r="A49" s="21" t="inlineStr">
         <is>
           <t>4. MANUAL OVERRIDES  (escape hatch)</t>
         </is>
@@ -26264,133 +27842,133 @@
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="20" t="inlineStr">
+      <c r="A54" s="21" t="inlineStr">
         <is>
           <t>5. WORKED EXAMPLE: Phoveus (Attacker) vs Harith (Defender)</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
-      <c r="A56" s="21" t="inlineStr">
+      <c r="A56" s="20" t="inlineStr">
         <is>
           <t>Role Advantage: Fighter vs Mage = +1 x role_mult(5) = 5</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
-      <c r="A57" s="21" t="inlineStr">
+      <c r="A57" s="20" t="inlineStr">
         <is>
           <t>Stat: ((70+30)/2 − 40) x burst_mult(0.1) = 1</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
-      <c r="A58" s="21" t="inlineStr">
+      <c r="A58" s="20" t="inlineStr">
         <is>
           <t>Difficulty Gap: (30−50) is not &gt;20, so = 0</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
-      <c r="A59" s="21" t="inlineStr">
+      <c r="A59" s="20" t="inlineStr">
         <is>
           <t>Damage Type Advantage: Phoveus = Mixed → dmgtype_mixed = 5</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
-      <c r="A60" s="21" t="inlineStr">
+      <c r="A60" s="20" t="inlineStr">
         <is>
           <t>Power Spike Timing: (3−3) x spike_mult(3) = 0</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
-      <c r="A61" s="21" t="inlineStr">
+      <c r="A61" s="20" t="inlineStr">
         <is>
           <t>Style Matchup: Phoveus(Shield/Burst) vs Harith(Shield/Dash-Blink) best cell = 0</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
-      <c r="A62" s="21" t="inlineStr">
+      <c r="A62" s="20" t="inlineStr">
         <is>
           <t>Hard Counter Bonus: Harith is tagged Dash/Blink → Phoveus rule fires: 18 − (−25) = 43</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
-      <c r="A63" s="21" t="inlineStr">
+      <c r="A63" s="20" t="inlineStr">
         <is>
           <t>TOTAL = 5+1+0+5+0+0+43 = 54  → Phoveus ranks #1 counter for Harith in the Lookup sheet.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="20" t="inlineStr">
+      <c r="A65" s="21" t="inlineStr">
         <is>
           <t>6. WORKED EXAMPLE: Faramis (Attacker) vs Gloo (Defender)</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
-      <c r="A67" s="21" t="inlineStr">
+      <c r="A67" s="20" t="inlineStr">
         <is>
           <t>Role Advantage: Support vs Tank = -1, but role2 Mage vs Tank = +1 → MAX = +1 x role_mult(5) = 5</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
-      <c r="A68" s="21" t="inlineStr">
+      <c r="A68" s="20" t="inlineStr">
         <is>
           <t>Stat: ((60+10)/2 − 100) x 0.1 = -6.5</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
-      <c r="A69" s="21" t="inlineStr">
+      <c r="A69" s="20" t="inlineStr">
         <is>
           <t>Difficulty Gap: (40−70) not &gt;20 → 0</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
-      <c r="A70" s="21" t="inlineStr">
+      <c r="A70" s="20" t="inlineStr">
         <is>
           <t>Damage Type Advantage: both Magic → dmgtype_same = -2</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
-      <c r="A71" s="21" t="inlineStr">
+      <c r="A71" s="20" t="inlineStr">
         <is>
           <t>Power Spike Timing: (5−2) x 3 = 9</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
-      <c r="A72" s="21" t="inlineStr">
+      <c r="A72" s="20" t="inlineStr">
         <is>
           <t>Style Matchup: best cell among Faramis(Healing/AoE Damage) vs Gloo(Sustain/Targeted CC) = 0</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
-      <c r="A73" s="21" t="inlineStr">
+      <c r="A73" s="20" t="inlineStr">
         <is>
           <t>Hard Counter Bonus: Faramis | Hero | Gloo rule fires: 20 − (−18) = 38</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
-      <c r="A74" s="21" t="inlineStr">
+      <c r="A74" s="20" t="inlineStr">
         <is>
           <t>TOTAL = 5 − 6.5 + 0 − 2 + 9 + 0 + 38 = 43.5  → Faramis ranks #1 counter for Gloo in the Lookup sheet.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="20" t="inlineStr">
+      <c r="A76" s="21" t="inlineStr">
         <is>
           <t>7. EDITING CHECKLIST</t>
         </is>
@@ -26454,20 +28032,21 @@
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="A17:J17"/>
     <mergeCell ref="A62:J62"/>
+    <mergeCell ref="A29:J29"/>
     <mergeCell ref="A35:J35"/>
-    <mergeCell ref="A29:J29"/>
-    <mergeCell ref="A81:J81"/>
+    <mergeCell ref="A33:J33"/>
+    <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A38:J38"/>
     <mergeCell ref="A43:J43"/>
-    <mergeCell ref="A38:J38"/>
     <mergeCell ref="A72:J72"/>
     <mergeCell ref="A52:J52"/>
-    <mergeCell ref="A20:J20"/>
     <mergeCell ref="A10:J10"/>
+    <mergeCell ref="A81:J81"/>
+    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A44:J44"/>
+    <mergeCell ref="A63:J63"/>
     <mergeCell ref="A68:J68"/>
-    <mergeCell ref="A63:J63"/>
-    <mergeCell ref="A44:J44"/>
-    <mergeCell ref="A19:J19"/>
-    <mergeCell ref="A13:J13"/>
     <mergeCell ref="A58:J58"/>
     <mergeCell ref="A9:J9"/>
     <mergeCell ref="A67:J67"/>
@@ -26476,16 +28055,16 @@
     <mergeCell ref="A83:J83"/>
     <mergeCell ref="A15:J15"/>
     <mergeCell ref="A59:J59"/>
+    <mergeCell ref="A24:J24"/>
     <mergeCell ref="A73:J73"/>
-    <mergeCell ref="A24:J24"/>
     <mergeCell ref="A82:J82"/>
     <mergeCell ref="A60:J60"/>
+    <mergeCell ref="A11:J11"/>
     <mergeCell ref="A49:J49"/>
     <mergeCell ref="A51:J51"/>
-    <mergeCell ref="A11:J11"/>
     <mergeCell ref="A45:J45"/>
+    <mergeCell ref="A36:J36"/>
     <mergeCell ref="A79:J79"/>
-    <mergeCell ref="A36:J36"/>
     <mergeCell ref="A61:J61"/>
     <mergeCell ref="A70:J70"/>
     <mergeCell ref="A78:J78"/>
@@ -26497,23 +28076,22 @@
     <mergeCell ref="A80:J80"/>
     <mergeCell ref="A46:J46"/>
     <mergeCell ref="A84:J84"/>
-    <mergeCell ref="A71:J71"/>
     <mergeCell ref="A74:J74"/>
     <mergeCell ref="A56:J56"/>
     <mergeCell ref="A27:J27"/>
     <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A26:J26"/>
     <mergeCell ref="A57:J57"/>
-    <mergeCell ref="A26:J26"/>
     <mergeCell ref="A42:J42"/>
     <mergeCell ref="A76:J76"/>
-    <mergeCell ref="A33:J33"/>
+    <mergeCell ref="A71:J71"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27005,7 +28583,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27167,7 +28745,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>